<commit_message>
Add initial documentation and project structure for A-Star-DUSt3R
- Created various markdown files for paper contributions, glossary, limitations, summary, references, and related work.
- Established technical documentation including architecture, evaluation, experiments, implementation, inference, mathematical formulation, pipeline, and training.
- Developed video planning documents such as animation plan, asset list, scene list, storyboard, and voice script.
- Organized project notes and guidelines for team collaboration and project execution.
- Added placeholder Python scripts for video scenes and utility functions.
- Included a BibTeX file and placeholder PDFs for references.
</commit_message>
<xml_diff>
--- a/project/[FAI] Project 2526-3.xlsx
+++ b/project/[FAI] Project 2526-3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="202">
   <si>
     <t>Dấu thời gian</t>
   </si>
@@ -469,7 +469,154 @@
     <t>openaccess.thecvf.com</t>
   </si>
   <si>
+    <t>pqtuan19@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>A-Star</t>
+  </si>
+  <si>
+    <t>DUSt3R: Geometric 3D Vision Made Easy</t>
+  </si>
+  <si>
+    <t>https://openaccess.thecvf.com/content/CVPR2024/html/Wang_DUSt3R_Geometric_3D_Vision_Made_Easy_CVPR_2024_paper.html</t>
+  </si>
+  <si>
+    <t>lmhoang18@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>Max Verstappen</t>
+  </si>
+  <si>
+    <t>Gaussian Splatting SLAM</t>
+  </si>
+  <si>
+    <t>https://openaccess.thecvf.com/content/CVPR2024/html/Matsuki_Gaussian_Splatting_SLAM_CVPR_2024_paper.html</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2312.06741</t>
+  </si>
+  <si>
+    <t>cdvan2427@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>Satellite Videos Object Tracking Based on Enhanced Correlation Filter With Motion Prediction Network</t>
+  </si>
+  <si>
+    <t>IEEE Journal of Selected Topics in Applied Earth Observations and Remote Sensing</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/10582298</t>
+  </si>
+  <si>
+    <t>https://wos-journal.info/journalid/13537</t>
+  </si>
+  <si>
     <t>Reviewing</t>
+  </si>
+  <si>
+    <t>nhghieu22@clc.fitus.edu.vnn</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>3D Gaussian Splatting for Real-Time Radiance Field Rendering</t>
+  </si>
+  <si>
+    <t>ACM Transactions on Graphics, Association for Computing Machinery</t>
+  </si>
+  <si>
+    <t>https://dl.acm.org/doi/10.1145/3592433</t>
+  </si>
+  <si>
+    <t>https://wos-journal.info/journalid/563</t>
+  </si>
+  <si>
+    <t>ngcu2421@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>MU</t>
+  </si>
+  <si>
+    <t>LightGlue: Local Feature Matching at Light Speed</t>
+  </si>
+  <si>
+    <t>International Conference on Computer Vision (ICCV)</t>
+  </si>
+  <si>
+    <t>https://openaccess.thecvf.com/content/ICCV2023/html/Lindenberger_LightGlue_Local_Feature_Matching_at_Light_Speed_ICCV_2023_paper.html</t>
+  </si>
+  <si>
+    <t>https://portal.core.edu.au/conf-ranks/638/</t>
+  </si>
+  <si>
+    <t>dlplinh2414@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>SVT</t>
+  </si>
+  <si>
+    <t>OpenVLA: An Open-Source Vision-Language-Action Model</t>
+  </si>
+  <si>
+    <t>https://openreview.net/forum?id=ZMnD6QZAE6</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2406.09246</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/scholar?as_vis=1&amp;q=OpenVLA:+An+Open-Source+Vision-Language-Action+Model&amp;hl=vi&amp;as_sdt=0,5</t>
+  </si>
+  <si>
+    <t>npmng2413@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>NKT</t>
+  </si>
+  <si>
+    <t>VoxPoser: Composable 3D Value Maps for Robotic Manipulation with Language Models</t>
+  </si>
+  <si>
+    <t>https://proceedings.mlr.press/v229/huang23b.html</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/scholar?cites=7844573100140075704&amp;as_sdt=2005&amp;sciodt=0,5&amp;hl=vi</t>
+  </si>
+  <si>
+    <t>Ghi nhầm tháng - venue?</t>
+  </si>
+  <si>
+    <t>nthtruc2411@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>Ctrl+AI</t>
+  </si>
+  <si>
+    <t>MVTracker: Multi-View 3D Point Tracking</t>
+  </si>
+  <si>
+    <t>IEEE/CVF International Conference on Computer Vision (ICCV)</t>
+  </si>
+  <si>
+    <t>https://openaccess.thecvf.com/content/ICCV2025/html/Rajic_Multi-View_3D_Point_Tracking_ICCV_2025_paper.html</t>
+  </si>
+  <si>
+    <t>nkngan2411@clc.fitus.edu.vn</t>
+  </si>
+  <si>
+    <t>NeuroCore</t>
+  </si>
+  <si>
+    <t>YOLO-World: Real-Time Open-Vocabulary Object Detection</t>
+  </si>
+  <si>
+    <t>https://openaccess.thecvf.com/content/CVPR2024/html/Cheng_YOLO-World_Real-Time_Open-Vocabulary_Object_Detection_CVPR_2024_paper.html?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>https://openaccess.thecvf.com/content/CVPR2024/html/Cheng_YOLO-World_Real-Time_Open-Vocabulary_Object_Detection_CVPR_2024_paper.html</t>
+  </si>
+  <si>
+    <t>https://portal.core.edu.au/conf-ranks/</t>
   </si>
 </sst>
 </file>
@@ -639,7 +786,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:P25" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:P34" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="16">
     <tableColumn name="Dấu thời gian" id="1"/>
     <tableColumn name="Địa chỉ email" id="2"/>
@@ -967,7 +1114,7 @@
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10">
-        <f t="shared" ref="O2:O25" si="1">DATEDIF(DATE(F2, G2, 1), TODAY(), "M")</f>
+        <f t="shared" ref="O2:O34" si="1">DATEDIF(DATE(F2, G2, 1), TODAY(), "M")</f>
         <v>31</v>
       </c>
       <c r="P2" s="10">
@@ -2044,57 +2191,447 @@
       </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="13" t="s">
+      <c r="A25" s="5">
+        <v>46222.72094642361</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="N25" s="14"/>
-      <c r="O25" s="10" t="str">
+      <c r="C25" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F25" s="6">
+        <v>2024.0</v>
+      </c>
+      <c r="G25" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O25" s="10">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="P25" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="5">
+        <v>46224.39399327546</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="F26" s="6">
+        <v>2024.0</v>
+      </c>
+      <c r="G26" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M26" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O26" s="10">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="P26" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="5">
+        <v>46228.91422368056</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="F27" s="6">
+        <v>2024.0</v>
+      </c>
+      <c r="G27" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="M27" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="O27" s="10">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="P27" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="5">
+        <v>46229.59223394676</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="F28" s="6">
+        <v>2023.0</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="M28" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O28" s="10">
+        <f t="shared" si="1"/>
+        <v>43</v>
+      </c>
+      <c r="P28" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="5">
+        <v>46229.89215702546</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="F29" s="6">
+        <v>2023.0</v>
+      </c>
+      <c r="G29" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="M29" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O29" s="10">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="P29" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="5">
+        <v>46230.999148125</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F30" s="6">
+        <v>2024.0</v>
+      </c>
+      <c r="G30" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="K30" s="6">
+        <v>3345.0</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="M30" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O30" s="10">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="P30" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="5">
+        <v>46231.48326357639</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F31" s="6">
+        <v>2023.0</v>
+      </c>
+      <c r="H31" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="K31" s="6">
+        <v>1188.0</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="M31" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="O31" s="10">
+        <f t="shared" si="1"/>
+        <v>43</v>
+      </c>
+      <c r="P31" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="5">
+        <v>46232.96908201389</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F32" s="6">
+        <v>2025.0</v>
+      </c>
+      <c r="G32" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L32" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="M32" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O32" s="10">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="P32" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="5">
+        <v>46233.026380763884</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F33" s="6">
+        <v>2024.0</v>
+      </c>
+      <c r="G33" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="M33" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="O33" s="10">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="P33" s="10">
+        <f>Form_Responses[Month time]*2</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="12"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="N34" s="14"/>
+      <c r="O34" s="10" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="P25" s="12" t="str">
+      <c r="P34" s="12" t="str">
         <f>Form_Responses[Month time]*2</f>
         <v>#NUM!</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="N26" s="15"/>
-    </row>
-    <row r="27">
-      <c r="N27" s="15"/>
-    </row>
-    <row r="28">
-      <c r="N28" s="15"/>
-    </row>
-    <row r="29">
-      <c r="N29" s="15"/>
-    </row>
-    <row r="30">
-      <c r="N30" s="15"/>
-    </row>
-    <row r="31">
-      <c r="N31" s="15"/>
-    </row>
-    <row r="32">
-      <c r="N32" s="15"/>
-    </row>
-    <row r="33">
-      <c r="N33" s="15"/>
-    </row>
-    <row r="34">
-      <c r="N34" s="15"/>
     </row>
     <row r="35">
       <c r="N35" s="15"/>
@@ -2366,9 +2903,36 @@
     <row r="124">
       <c r="N124" s="15"/>
     </row>
+    <row r="125">
+      <c r="N125" s="15"/>
+    </row>
+    <row r="126">
+      <c r="N126" s="15"/>
+    </row>
+    <row r="127">
+      <c r="N127" s="15"/>
+    </row>
+    <row r="128">
+      <c r="N128" s="15"/>
+    </row>
+    <row r="129">
+      <c r="N129" s="15"/>
+    </row>
+    <row r="130">
+      <c r="N130" s="15"/>
+    </row>
+    <row r="131">
+      <c r="N131" s="15"/>
+    </row>
+    <row r="132">
+      <c r="N132" s="15"/>
+    </row>
+    <row r="133">
+      <c r="N133" s="15"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="M2:M25">
+    <dataValidation type="list" allowBlank="1" sqref="M2:M34">
       <formula1>"Accepted,Rejected,Reviewing"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2430,10 +2994,31 @@
     <hyperlink r:id="rId55" ref="I24"/>
     <hyperlink r:id="rId56" ref="J24"/>
     <hyperlink r:id="rId57" ref="L24"/>
+    <hyperlink r:id="rId58" ref="I25"/>
+    <hyperlink r:id="rId59" ref="L25"/>
+    <hyperlink r:id="rId60" ref="I26"/>
+    <hyperlink r:id="rId61" ref="J26"/>
+    <hyperlink r:id="rId62" ref="L26"/>
+    <hyperlink r:id="rId63" ref="I27"/>
+    <hyperlink r:id="rId64" ref="L27"/>
+    <hyperlink r:id="rId65" ref="I28"/>
+    <hyperlink r:id="rId66" ref="L28"/>
+    <hyperlink r:id="rId67" ref="I29"/>
+    <hyperlink r:id="rId68" ref="L29"/>
+    <hyperlink r:id="rId69" ref="I30"/>
+    <hyperlink r:id="rId70" ref="J30"/>
+    <hyperlink r:id="rId71" ref="L30"/>
+    <hyperlink r:id="rId72" ref="I31"/>
+    <hyperlink r:id="rId73" ref="L31"/>
+    <hyperlink r:id="rId74" ref="I32"/>
+    <hyperlink r:id="rId75" ref="L32"/>
+    <hyperlink r:id="rId76" ref="H33"/>
+    <hyperlink r:id="rId77" ref="I33"/>
+    <hyperlink r:id="rId78" ref="L33"/>
   </hyperlinks>
-  <drawing r:id="rId58"/>
+  <drawing r:id="rId79"/>
   <tableParts count="1">
-    <tablePart r:id="rId60"/>
+    <tablePart r:id="rId81"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>